<commit_message>
Clear validation rules and add signal diagnostic logging
- Remove all validation rule rows from quick_demo/v1.0
  validation_rules_sheet.xlsx (ring numbers were stale for
  the current chip).
- Add diagnostic logging to _compute_signal and
  _find_step_row to trace step lookup, time window, and
  signal collection for debugging hsCRP analysis.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/config/calibration_data/quick_demo/v1.0/validation_rules_sheet.xlsx
+++ b/config/calibration_data/quick_demo/v1.0/validation_rules_sheet.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -481,111 +481,6 @@
       <c r="M1" t="inlineStr">
         <is>
           <t>Assay specific</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Neg ctrl rings between -50 and 100 pm net shift</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Signal difference</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Net shift</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>TIMING: cart_dispense_GNP (start)</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>5</v>
-      </c>
-      <c r="F2" t="n">
-        <v>30</v>
-      </c>
-      <c r="G2" t="n">
-        <v>-50</v>
-      </c>
-      <c r="H2" t="n">
-        <v>100</v>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>3,14</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>3,14</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>hsCRP</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>CRP rings greater than -20 pm net shift</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Signal difference</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Net shift</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>TIMING: cart_dispense_GNP (start)</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>5</v>
-      </c>
-      <c r="F3" t="n">
-        <v>30</v>
-      </c>
-      <c r="G3" t="n">
-        <v>-20</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>4,11</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>4,11</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>hsCRP</t>
         </is>
       </c>
     </row>
@@ -645,7 +540,6 @@
           <t>R-Squared</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -653,7 +547,6 @@
           <t>Pearson R</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -661,7 +554,6 @@
           <t>Slope</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -669,7 +561,6 @@
           <t>Number of points</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -677,7 +568,6 @@
           <t>Change in slope</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -685,7 +575,6 @@
           <t>CV</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -693,7 +582,6 @@
           <t>No rule</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -701,7 +589,6 @@
           <t>RMSD of slope</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -709,7 +596,6 @@
           <t>MAD of slope</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>